<commit_message>
Ajuste no notebook para correção de bug
</commit_message>
<xml_diff>
--- a/data/predictions/botafogo_previsao_estadio.xlsx
+++ b/data/predictions/botafogo_previsao_estadio.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30305"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30318"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9399af9f441dfb25/Documentos/Projeto Futebol/ia-botafogo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5668" documentId="8_{FF0F605F-F2C5-4D0A-9132-A4D8069F1A8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88B259E8-0282-4014-95A8-72B0595C3B96}"/>
+  <xr:revisionPtr revIDLastSave="5678" documentId="8_{FF0F605F-F2C5-4D0A-9132-A4D8069F1A8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6DAC19AF-10DA-46A7-A95B-DBAC9E503E7F}"/>
   <bookViews>
     <workbookView minimized="1" xWindow="2268" yWindow="2268" windowWidth="17280" windowHeight="8880" xr2:uid="{BDAF93C4-966A-4323-BFDC-13327AEDDB19}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2283" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2284" uniqueCount="173">
   <si>
     <t>ano_campeonato</t>
   </si>
@@ -19416,6 +19416,21 @@
       <c r="L303">
         <v>46931</v>
       </c>
+      <c r="M303">
+        <v>457870</v>
+      </c>
+      <c r="N303">
+        <v>538867.56000000006</v>
+      </c>
+      <c r="O303">
+        <v>1400.3</v>
+      </c>
+      <c r="P303">
+        <v>-80997.56</v>
+      </c>
+      <c r="Q303">
+        <v>-80997.56</v>
+      </c>
       <c r="S303" t="s">
         <v>35</v>
       </c>
@@ -19463,9 +19478,18 @@
       <c r="F304" s="3">
         <v>0.8125</v>
       </c>
+      <c r="G304">
+        <v>22</v>
+      </c>
+      <c r="H304">
+        <v>2</v>
+      </c>
       <c r="I304">
         <v>4</v>
       </c>
+      <c r="J304" t="s">
+        <v>44</v>
+      </c>
       <c r="L304">
         <v>46931</v>
       </c>
@@ -19480,6 +19504,9 @@
       </c>
       <c r="X304" t="s">
         <v>167</v>
+      </c>
+      <c r="Y304">
+        <v>5</v>
       </c>
       <c r="Z304">
         <v>9</v>
@@ -19531,7 +19558,7 @@
         <v>46232</v>
       </c>
       <c r="H306">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I306">
         <v>21</v>

</xml_diff>